<commit_message>
Update data.xlsx with new content
</commit_message>
<xml_diff>
--- a/src/ainnovation/data/data.xlsx
+++ b/src/ainnovation/data/data.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Alo tudo bem  preciso que me ma" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Sheet1" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="areas" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="curso " sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -29,19 +29,25 @@
     <t>Descrição com Palavras-Chave</t>
   </si>
   <si>
+    <t>Interesse &amp; Motivação</t>
+  </si>
+  <si>
     <t>Link Oficial da Faculdade</t>
   </si>
   <si>
-    <t>Interesse &amp; Motivação</t>
+    <t>Competências Desenvolvidas</t>
   </si>
   <si>
     <t>Universidade dos Açores</t>
   </si>
   <si>
+    <t>Tipo de Trabalho Esperado</t>
+  </si>
+  <si>
     <t>Faculdade de Ciências Agrárias e do Ambiente</t>
   </si>
   <si>
-    <t>Competências Desenvolvidas</t>
+    <t>Estilo de Aprendizagem</t>
   </si>
   <si>
     <t>Licenciatura e Mestrado (2º Ciclo)</t>
@@ -50,19 +56,19 @@
     <t>Ciências da Saúde e Biológicas, Artes, Património e Agricultura, Ciências do Mar e Ambiente, Biotecnologia, Veterinária, Insularidade</t>
   </si>
   <si>
-    <t>Tipo de Trabalho Esperado</t>
+    <t>Vantagens / Oportunidades</t>
   </si>
   <si>
     <t>UAc - FCAA</t>
   </si>
   <si>
-    <t>Estilo de Aprendizagem</t>
+    <t>Desvantagens / Desafios</t>
   </si>
   <si>
     <t>Faculdade de Ciências Sociais e Humanas</t>
   </si>
   <si>
-    <t>Vantagens / Oportunidades</t>
+    <t>Dúvidas a Esclarecer / Pontos Críticos</t>
   </si>
   <si>
     <t>Humanidades e Letras, Ciências Sociais e Comunicação, Estudos Europeus, História, Línguas, Cultura atlântica</t>
@@ -71,103 +77,121 @@
     <t>UAc - FCSH</t>
   </si>
   <si>
-    <t>Desvantagens / Desafios</t>
-  </si>
-  <si>
     <t>Faculdade de Ciências e Tecnologia</t>
   </si>
   <si>
-    <t>Dúvidas a Esclarecer / Pontos Críticos</t>
-  </si>
-  <si>
     <t>Ciências Exatas e Tecnologias, Engenharia e Tecnologias, Investigação científica, Tecnologias, Biodiversidade</t>
   </si>
   <si>
     <t>UAc - FCT</t>
   </si>
   <si>
+    <t>Faculdade de Economia e Gestão</t>
+  </si>
+  <si>
+    <t>Gestão e Economia, Ciências Empresariais e Direito, Finanças, Mercados, Empreendedorismo</t>
+  </si>
+  <si>
+    <t>UAc - FEG</t>
+  </si>
+  <si>
+    <t>Escola Superior de Saúde - Ponta Delgada / Angra</t>
+  </si>
+  <si>
+    <t>Licenciatura</t>
+  </si>
+  <si>
+    <t>Ciências da Saúde e Biológicas, Enfermagem, Cuidados de saúde, Clínico, Bem-estar</t>
+  </si>
+  <si>
+    <t>UAc - ESS</t>
+  </si>
+  <si>
+    <t>Universidade do Algarve</t>
+  </si>
+  <si>
     <t>Engenharia e Tecnologias</t>
   </si>
   <si>
-    <t>Faculdade de Economia e Gestão</t>
-  </si>
-  <si>
-    <t>Gestão e Economia, Ciências Empresariais e Direito, Finanças, Mercados, Empreendedorismo</t>
-  </si>
-  <si>
-    <t>UAc - FEG</t>
-  </si>
-  <si>
     <t>Alta empregabilidade e inovação tecnológica</t>
   </si>
   <si>
+    <t>Ciências do Mar e Ambiente, Engenharia e Tecnologias, Ciências Exatas, Oceanografia, Gestão costeira</t>
+  </si>
+  <si>
     <t>Resolução de problemas complexos, Programação, Análise</t>
   </si>
   <si>
-    <t>Escola Superior de Saúde - Ponta Delgada / Angra</t>
+    <t>UAlg - FCT</t>
   </si>
   <si>
     <t>Trabalho de projeto, R&amp;D, Consultoria técnica</t>
   </si>
   <si>
-    <t>Licenciatura</t>
-  </si>
-  <si>
     <t>Teórico-prático, Laboratorial intensivo</t>
   </si>
   <si>
-    <t>Ciências da Saúde e Biológicas, Enfermagem, Cuidados de saúde, Clínico, Bem-estar</t>
-  </si>
-  <si>
-    <t>UAc - ESS</t>
-  </si>
-  <si>
-    <t>Alta empregabilidade, salários competitivos, facilidade de trabalho remoto e internacional.</t>
-  </si>
-  <si>
-    <t>Ritmo de atualização tecnológica muito rápido (risco de obsolescência), stresse em projetos críticos.</t>
-  </si>
-  <si>
-    <t>Universidade do Algarve</t>
+    <t>Faculdade de Economia</t>
+  </si>
+  <si>
+    <t>Alta procura no mercado, forte propensão para trabalho remoto e oportunidades internacionais.</t>
+  </si>
+  <si>
+    <t>Gestão e Economia, Ciências Empresariais e Direito, Finanças globais, Análise económica, Negócios</t>
+  </si>
+  <si>
+    <t>UAlg - FE</t>
+  </si>
+  <si>
+    <t>Ritmo de atualização tecnológica muito rápido (risco de obsolescência de competências), stresse em projetos críticos.</t>
+  </si>
+  <si>
+    <t>Faculdade de Ciências Humanas e Sociais</t>
   </si>
   <si>
     <t>O curso exige bases de matemática muito fortes no 1º ano? Qual a percentagem de aulas teóricas vs. projeto prático?</t>
   </si>
   <si>
+    <t>Ciências Sociais e Comunicação, Humanidades e Letras, Línguas, Património, Comunicação estratégica</t>
+  </si>
+  <si>
+    <t>UAlg - FCHS</t>
+  </si>
+  <si>
     <t>Ciências da Saúde e Biológicas</t>
   </si>
   <si>
-    <t>Ciências do Mar e Ambiente, Engenharia e Tecnologias, Ciências Exatas, Oceanografia, Gestão costeira</t>
-  </si>
-  <si>
     <t>Investigação médica e impacto social</t>
   </si>
   <si>
-    <t>UAlg - FCT</t>
+    <t>Faculdade de Medicina e Ciências Biomédicas</t>
   </si>
   <si>
     <t>Pensamento crítico, Investigação laboratorial, Ética</t>
   </si>
   <si>
+    <t>Mestrado Integrado e 2º Ciclo</t>
+  </si>
+  <si>
     <t>Clínico, Investigação científica, Indústria farmacêutica</t>
   </si>
   <si>
-    <t>Faculdade de Economia</t>
+    <t>Ciências da Saúde e Biológicas, Investigação médica, Clínico, Ciências da vida, Saúde humana</t>
   </si>
   <si>
     <t>Prático em laboratório/hospital, Autodidata</t>
   </si>
   <si>
-    <t>Alto impacto social, empregabilidade estável, forte reconhecimento profissional.</t>
-  </si>
-  <si>
-    <t>Gestão e Economia, Ciências Empresariais e Direito, Finanças globais, Análise económica, Negócios</t>
+    <t>UAlg - FMCB</t>
+  </si>
+  <si>
+    <t>Alto impacto social, perspetivas de estabilidade profissional e forte reconhecimento na sociedade.</t>
   </si>
   <si>
     <t>Cursos longos e exigentes (mestrados integrados pesados), turnos e horários complexos no mercado.</t>
   </si>
   <si>
-    <t>UAlg - FE</t>
+    <t>Instituto Superior de Engenharia</t>
   </si>
   <si>
     <t>Quais são as saídas profissionais exatas fora da investigação pura? Os estágios clínicos começam em que ano?</t>
@@ -179,103 +203,100 @@
     <t>Paixão por cultura, línguas e história</t>
   </si>
   <si>
-    <t>Faculdade de Ciências Humanas e Sociais</t>
+    <t>Engenharia e Tecnologias, Ciências Exatas e Tecnologias, Eletrónica, Civil, Mecânica, Sistemas</t>
   </si>
   <si>
     <t>Comunicação avançada, Pensamento crítico, Escrita</t>
   </si>
   <si>
+    <t>UAlg - ISE</t>
+  </si>
+  <si>
     <t>Ensino, Tradução, Gestão cultural, Investigação</t>
   </si>
   <si>
-    <t>Ciências Sociais e Comunicação, Humanidades e Letras, Línguas, Património, Comunicação estratégica</t>
-  </si>
-  <si>
     <t>Leitura intensiva, Debate académico, Aulas magistrais</t>
   </si>
   <si>
-    <t>UAlg - FCHS</t>
+    <t>Escola Superior de Gestão, Hotelaria e Turismo</t>
   </si>
   <si>
     <t>Desenvolvimento profundo de pensamento crítico, empatia cultural e excelentes capacidades de comunicação.</t>
   </si>
   <si>
-    <t>Faculdade de Medicina e Ciências Biomédicas</t>
-  </si>
-  <si>
-    <t>Empregabilidade inicial desafiante em Portugal, menor previsibilidade salarial de entrada.</t>
-  </si>
-  <si>
-    <t>Mestrado Integrado e 2º Ciclo</t>
-  </si>
-  <si>
-    <t>Que tipo de saídas profissionais existem além da docência? É necessário tirar mestrado obrigatoriamente para ter emprego estável?</t>
-  </si>
-  <si>
-    <t>Ciências da Saúde e Biológicas, Investigação médica, Clínico, Ciências da vida, Saúde humana</t>
-  </si>
-  <si>
-    <t>UAlg - FMCB</t>
+    <t>Inserção profissional inicial desafiante em Portugal.</t>
+  </si>
+  <si>
+    <t>Que tipo de saídas profissionais existem além da docência? É necessário tirar mestrado obrigatoriamente para ter estabilidade?</t>
   </si>
   <si>
     <t>Gestão e Economia</t>
   </si>
   <si>
+    <t>Gestão e Economia, Turismo, Hotelaria, Gestão turística, Ecoturismo</t>
+  </si>
+  <si>
     <t>Empreendedorismo, finanças e liderança de mercado</t>
   </si>
   <si>
+    <t>UAlg - ESGHT</t>
+  </si>
+  <si>
     <t>Liderança, Negociação, Análise de dados financeiros</t>
   </si>
   <si>
-    <t>Instituto Superior de Engenharia</t>
-  </si>
-  <si>
     <t>Corporativo, Consultoria de gestão, Startups</t>
   </si>
   <si>
+    <t>Escola Superior de Saúde</t>
+  </si>
+  <si>
     <t>Casos de estudo práticos, Trabalho de equipa</t>
   </si>
   <si>
-    <t>Versatilidade corporativa, excelentes redes de contactos (networking), progressão rápida de carreira.</t>
-  </si>
-  <si>
-    <t>Engenharia e Tecnologias, Ciências Exatas e Tecnologias, Eletrónica, Civil, Mecânica, Sistemas</t>
+    <t>Versatilidade corporativa, excelentes redes de contactos (networking) e perspetiva de progressão de carreira.</t>
+  </si>
+  <si>
+    <t>Ciências da Saúde e Biológicas, Enfermagem, Tecnologias da saúde, Fisioterapia</t>
   </si>
   <si>
     <t>Alta concorrência inicial no mercado de trabalho, pressão constante por resultados e metas.</t>
   </si>
   <si>
-    <t>UAlg - ISE</t>
+    <t>UAlg - ESS</t>
   </si>
   <si>
     <t>O curso foca-se mais em teoria económica ou em ferramentas práticas de negócio e software de gestão?</t>
   </si>
   <si>
-    <t>Escola Superior de Gestão, Hotelaria e Turismo</t>
+    <t>Escola Superior de Educação e Comunicação</t>
   </si>
   <si>
     <t>Tecnologias e Design</t>
   </si>
   <si>
+    <t>Ciências Sociais e Comunicação, Psicologia e Ciências da Educação, Ensino, Multimédia</t>
+  </si>
+  <si>
     <t>Criatividade aplicada à tecnologia e inovação</t>
   </si>
   <si>
-    <t>Gestão e Economia, Turismo, Hotelaria, Gestão turística, Ecoturismo</t>
+    <t>UAlg - ESEC</t>
   </si>
   <si>
     <t>Design thinking, Prototipagem, Engenharia criativa</t>
   </si>
   <si>
-    <t>UAlg - ESGHT</t>
-  </si>
-  <si>
     <t>Indústria criativa, Desenvolvimento de produto, UX/UI</t>
   </si>
   <si>
+    <t>Universidade de Aveiro</t>
+  </si>
+  <si>
     <t>Projeto prático contínuo, Aprendizagem baseada em projetos</t>
   </si>
   <si>
-    <t>Escola Superior de Saúde</t>
+    <t>Departamento / Escola Politécnica de Aveiro</t>
   </si>
   <si>
     <t>Combinação perfeita entre arte e lógica tecnológica, grande autonomia criativa em projetos.</t>
@@ -284,169 +305,226 @@
     <t>Saturação inicial no mercado de entrada para cargos juniores de design, necessidade de portefólio forte.</t>
   </si>
   <si>
-    <t>Ciências da Saúde e Biológicas, Enfermagem, Tecnologias da saúde, Fisioterapia</t>
-  </si>
-  <si>
     <t>Como é avaliado o trabalho prático? O foco é mais em prototipagem industrial ou em experiências digitais (UI/UX)?</t>
   </si>
   <si>
-    <t>UAlg - ESS</t>
+    <t>Engenharia e Tecnologias, Ciências Exatas, Tecnologias e Design, Investigação industrial, Inovação</t>
+  </si>
+  <si>
+    <t>UA - UA.pt</t>
+  </si>
+  <si>
+    <t>Escola Superior de Design, Gestão e Tecnologia (Águeda)</t>
   </si>
   <si>
     <t>Ciências Exatas e Tecnologias</t>
   </si>
   <si>
-    <t>Escola Superior de Educação e Comunicação</t>
+    <t>Tecnologias e Design, Gestão e Economia, Engenharia prática, Desenvolvimento de produto, Inovação</t>
   </si>
   <si>
     <t>Sustentabilidade, energias e inovação industrial</t>
   </si>
   <si>
+    <t>UA - ESTGA</t>
+  </si>
+  <si>
     <t>Engenharia prática, Sustentabilidade, Investigação aplicada</t>
   </si>
   <si>
-    <t>Ciências Sociais e Comunicação, Psicologia e Ciências da Educação, Ensino, Multimédia</t>
+    <t>Instituto Superior de Contabilidade e Administração</t>
   </si>
   <si>
     <t>Indústria, Gestão ambiental, Engenharia de processos</t>
   </si>
   <si>
-    <t>UAlg - ESEC</t>
-  </si>
-  <si>
     <t>Metodologia interdisciplinar, Forte componente prática</t>
   </si>
   <si>
-    <t>Universidade de Aveiro</t>
+    <t>Gestão e Economia, Ciências Empresariais e Direito, Contabilidade, Finanças, Auditoria</t>
+  </si>
+  <si>
+    <t>UA - ISCA</t>
   </si>
   <si>
     <t>Forte contributo para a transição energética e inovação industrial, relevância estratégica global.</t>
   </si>
   <si>
-    <t>Departamento / Escola Politécnica de Aveiro</t>
+    <t>Escola Superior de Saúde de Aveiro</t>
   </si>
   <si>
     <t>Dependência de investimento industrial e governamental em projetos de grande escala.</t>
   </si>
   <si>
-    <t>Quais são os setores industriais em Portugal que mais contratam este perfil específico?</t>
-  </si>
-  <si>
-    <t>Engenharia e Tecnologias, Ciências Exatas, Tecnologias e Design, Investigação industrial, Inovação</t>
+    <t>Ciências da Saúde e Biológicas, Enfermagem, Tecnologias da saúde, Diagnóstico, Clínico</t>
+  </si>
+  <si>
+    <t>Quais são os setores industriais em Portugal que mais absorvem este perfil específico?</t>
+  </si>
+  <si>
+    <t>UA - ESSA</t>
+  </si>
+  <si>
+    <t>Universidade da Beira Interior</t>
+  </si>
+  <si>
+    <t>UBI (Faculdades de Engenharia, Ciências, Artes, Letras, Sociais e Saúde)</t>
+  </si>
+  <si>
+    <t>Licenciatura, Mestrado Integrado e 2º Ciclo</t>
+  </si>
+  <si>
+    <t>Engenharia Aeroespacial e Tecnologias, Engenharia e Tecnologias, Ciências da Saúde, Artes Cinematográficas, Computação</t>
   </si>
   <si>
     <t>Direito e Políticas Públicas</t>
   </si>
   <si>
-    <t>UA - UA.pt</t>
+    <t>UBI</t>
   </si>
   <si>
     <t>Justiça, regulamentação e governação</t>
   </si>
   <si>
+    <t>Universidade de Coimbra</t>
+  </si>
+  <si>
+    <t>Faculdade de Direito</t>
+  </si>
+  <si>
     <t>Argumentação jurídica, Oratória, Análise legal</t>
   </si>
   <si>
-    <t>Escola Superior de Design, Gestão e Tecnologia (Águeda)</t>
+    <t>Direito e Políticas Públicas, Ciências Empresariais e Direito, Justiça, Regulamentação, Advocacia, Tradição legal</t>
   </si>
   <si>
     <t>Advocacia, Consultoria jurídica, Função pública</t>
   </si>
   <si>
+    <t>UC - FDUC</t>
+  </si>
+  <si>
     <t>Análise de jurisprudência, Debates, Memorandos</t>
   </si>
   <si>
-    <t>Tecnologias e Design, Gestão e Economia, Engenharia prática, Desenvolvimento de produto, Inovação</t>
+    <t>Faculdade de Letras</t>
   </si>
   <si>
     <t>Prestígio profissional, forte capacidade de argumentação e poder de decisão estrutural na sociedade.</t>
   </si>
   <si>
-    <t>UA - ESTGA</t>
-  </si>
-  <si>
-    <t>Mercado de advogados estagiários muito competitivo em Portugal, com retribuições iniciais baixas.</t>
+    <t>Humanidades e Letras, Património histórico, Investigação humanística, Línguas, Filosofia, Tradução</t>
+  </si>
+  <si>
+    <t>UC - FLUC</t>
+  </si>
+  <si>
+    <t>Mercado de estágio e início de carreira jurídico muito competitivo em Portugal, com retribuições iniciais modestas.</t>
   </si>
   <si>
     <t>Quais são as diferenças reais de saída entre seguir a carreira de Magistratura, Advocacia ou Consultoria Jurídica de Empresas?</t>
   </si>
   <si>
-    <t>Instituto Superior de Contabilidade e Administração</t>
+    <t>Engenharia e Tecnologias, Ciências Exatas e Tecnologias, Informática, Investigação científica, R&amp;D</t>
+  </si>
+  <si>
+    <t>UC - FCTUC</t>
+  </si>
+  <si>
+    <t>Faculdade de Medicina</t>
+  </si>
+  <si>
+    <t>Ciências da Saúde e Biológicas, Investigação médica, Clínico, Hospitais universitários, Ciências da vida</t>
   </si>
   <si>
     <t>Arquitetura e Urbanismo</t>
   </si>
   <si>
-    <t>Gestão e Economia, Ciências Empresariais e Direito, Contabilidade, Finanças, Auditoria</t>
+    <t>UC - FMUC</t>
   </si>
   <si>
     <t>Design de espaços e transformação urbana</t>
   </si>
   <si>
-    <t>UA - ISCA</t>
-  </si>
-  <si>
     <t>Criatividade espacial, Modelação 3D, Desenho técnico</t>
   </si>
   <si>
+    <t>Gestão e Economia, Ciências Sociais e Comunicação, Sociologia, Relações internacionais, Finanças</t>
+  </si>
+  <si>
+    <t>UC - FEUC</t>
+  </si>
+  <si>
     <t>Atelier de arquitetura, Planeamento urbano, Gestão de obra</t>
   </si>
   <si>
-    <t>Escola Superior de Saúde de Aveiro</t>
+    <t>Faculdade de Psicologia e de Ciências da Educação</t>
   </si>
   <si>
     <t>Estúdio criativo, Crítica contínua de projetos</t>
   </si>
   <si>
+    <t>Psicologia e Ciências da Educação, Comportamento humano, Diagnóstico comportamental, Pedagogia</t>
+  </si>
+  <si>
+    <t>UC - FPCEUC</t>
+  </si>
+  <si>
     <t>Realização pessoal tangível (ver o projeto construído), impacto direto na qualidade de vida urbana.</t>
   </si>
   <si>
-    <t>Ciências da Saúde e Biológicas, Enfermagem, Tecnologias da saúde, Diagnóstico, Clínico</t>
-  </si>
-  <si>
-    <t>UA - ESSA</t>
-  </si>
-  <si>
-    <t>Carga horária de projeto extremamente exigente (muitas noites em claro), custos altos com materiais e software.</t>
-  </si>
-  <si>
-    <t>Universidade da Beira Interior</t>
-  </si>
-  <si>
-    <t>Como funciona o acesso à Ordem dos Arquitetos após o mestrado? O estágio obrigatório é remunerado de forma justa?</t>
-  </si>
-  <si>
-    <t>UBI (Faculdades de Engenharia, Ciências, Artes, Letras, Sociais e Saúde)</t>
+    <t>Faculdade de Farmácia</t>
+  </si>
+  <si>
+    <t>Carga horária de projeto extremamente exigente (períodos intensos de trabalho), custos altos com materiais e software.</t>
+  </si>
+  <si>
+    <t>Ciências da Saúde e Biológicas, Ciências Farmacêuticas, Investigação laboratorial, Medicamentos</t>
+  </si>
+  <si>
+    <t>UC - FFUC</t>
+  </si>
+  <si>
+    <t>Como funciona o acesso à Ordem dos Arquitetos após o mestrado? O estágio obrigatório tem acompanhamento adequado?</t>
+  </si>
+  <si>
+    <t>Faculdade de Ciências do Desporto e Educação Física</t>
   </si>
   <si>
     <t>Ciências Sociais e Comunicação</t>
   </si>
   <si>
-    <t>Licenciatura, Mestrado Integrado e 2º Ciclo</t>
+    <t>Psicologia e Ciências da Educação, Desporto, Atividade física, Bem-estar, Motricidade</t>
   </si>
   <si>
     <t>Compreensão dos media, psicologia e sociedade</t>
   </si>
   <si>
-    <t>Engenharia Aeroespacial e Tecnologias, Engenharia e Tecnologias, Ciências da Saúde, Artes Cinematográficas, Computação</t>
+    <t>UC - FCDEF</t>
   </si>
   <si>
     <t>Comunicação estratégica, Empatia, Análise de dados sociais</t>
   </si>
   <si>
-    <t>UBI</t>
+    <t>Escola Superior de Enfermagem</t>
+  </si>
+  <si>
+    <t>Ciências da Saúde e Biológicas, Enfermagem, Cuidados de saúde, Prática clínica</t>
   </si>
   <si>
     <t>Media, Marketing, Recursos Humanos, ONG</t>
   </si>
   <si>
-    <t>Universidade de Coimbra</t>
+    <t>UC - ESEFDUC</t>
   </si>
   <si>
     <t>Seminários, Trabalho de campo, Ensino híbrido</t>
   </si>
   <si>
-    <t>Faculdade de Direito</t>
+    <t>Universidade de Évora</t>
+  </si>
+  <si>
+    <t>Escola de Ciências e Tecnologia</t>
   </si>
   <si>
     <t>Dinamismo profissional, versatilidade em agências, empresas ou comunicação institucional.</t>
@@ -455,64 +533,112 @@
     <t>Instabilidade laboral em alguns subsetores dos media tradicionais, forte dependência de tendências de mercado.</t>
   </si>
   <si>
-    <t>Direito e Políticas Públicas, Ciências Empresariais e Direito, Justiça, Regulamentação, Advocacia, Tradição legal</t>
-  </si>
-  <si>
-    <t>UC - FDUC</t>
-  </si>
-  <si>
-    <t>O curso dá mais peso ao jornalismo tradicional ou à comunicação digital, marketing de influência e gestão de redes?</t>
+    <t>Ciências Exatas e Tecnologias, Engenharia e Tecnologias, Ciências do Mar e Ambiente, Energias</t>
+  </si>
+  <si>
+    <t>UEvora - ECT</t>
+  </si>
+  <si>
+    <t>O curso dá mais peso ao jornalismo tradicional ou à comunicação digital, marketing e gestão de conteúdos?</t>
+  </si>
+  <si>
+    <t>Escola de Ciências Sociais</t>
+  </si>
+  <si>
+    <t>Ciências Sociais e Comunicação, Humanidades e Letras, Gestão e Economia, Sociologia, Educação</t>
+  </si>
+  <si>
+    <t>UEvora - ECS</t>
   </si>
   <si>
     <t>Engenharia Aeroespacial e Tecnologias</t>
   </si>
   <si>
-    <t>Faculdade de Letras</t>
+    <t>Escola de Artes</t>
   </si>
   <si>
     <t>Exploração do espaço, aeronáutica e mecânica</t>
   </si>
   <si>
+    <t>Artes, Património e Agricultura, Arquitetura e Urbanismo, Conservação e restauro, Design, Belas-Artes</t>
+  </si>
+  <si>
+    <t>UEvora - EA</t>
+  </si>
+  <si>
     <t>Cálculo avançado, Simulação de sistemas, Física aplicada</t>
   </si>
   <si>
-    <t>Humanidades e Letras, Património histórico, Investigação humanística, Línguas, Filosofia, Tradução</t>
+    <t>Escola de Saúde e Desenvolvimento Humano</t>
   </si>
   <si>
     <t>Indústria aeroespacial, Defesa, Investigação</t>
   </si>
   <si>
-    <t>UC - FLUC</t>
+    <t>Ciências da Saúde e Biológicas, Psicologia e Ciências da Educação, Enfermagem, Saúde, Bem-estar</t>
+  </si>
+  <si>
+    <t>UEvora - ESDH</t>
   </si>
   <si>
     <t>Prático, Simulações laboratoriais, Projetos de engenharia</t>
   </si>
   <si>
-    <t>Fascinio tecnológico de ponta, salários muito atrativos a nível internacional, alta valorização técnica.</t>
-  </si>
-  <si>
-    <t>Pouca expressão da indústria puramente aeroespacial em Portugal (muitos licenciados têm de emigrar).</t>
-  </si>
-  <si>
-    <t>Quais são as principais empresas ou agências internacionais onde os diplomados costumam conseguir colocação?</t>
-  </si>
-  <si>
-    <t>Engenharia e Tecnologias, Ciências Exatas e Tecnologias, Informática, Investigação científica, R&amp;D</t>
+    <t>Universidade da Madeira</t>
+  </si>
+  <si>
+    <t>Faculdade de Ciências Exatas e da Engenharia</t>
+  </si>
+  <si>
+    <t>Fascínio tecnológico de ponta, forte valorização técnica e analítica.</t>
+  </si>
+  <si>
+    <t>Engenharia e Tecnologias, Ciências Exatas e Tecnologias, Matemática, Computação, Engenharia</t>
+  </si>
+  <si>
+    <t>UMa - FCEE</t>
+  </si>
+  <si>
+    <t>Pouca expressão da indústria puramente aeroespacial em Portugal (muitos diplomados optam por oportunidades no estrangeiro).</t>
+  </si>
+  <si>
+    <t>Faculdade de Artes e Humanidades</t>
+  </si>
+  <si>
+    <t>Quais são as principais empresas ou centros internacionais onde os diplomados costumam conseguir colocação?</t>
+  </si>
+  <si>
+    <t>Humanidades e Letras, Artes, Património e Agricultura, Línguas, Cultura e turismo insular</t>
+  </si>
+  <si>
+    <t>UMa - FAH</t>
+  </si>
+  <si>
+    <t>Faculdade de Ciências Sociais</t>
   </si>
   <si>
     <t>Ciências do Mar e Ambiente</t>
   </si>
   <si>
-    <t>UC - FCTUC</t>
+    <t>Ciências Sociais e Comunicação, Gestão e Economia, Psicologia e Ciências da Educação, Direito</t>
+  </si>
+  <si>
+    <t>UMa - FCS</t>
   </si>
   <si>
     <t>Proteção dos oceanos, biologia marinha e turismo</t>
   </si>
   <si>
+    <t>Faculdade de Ciências da Vida</t>
+  </si>
+  <si>
     <t>Biologia de campo, Sustentabilidade, Gestão costeira</t>
   </si>
   <si>
-    <t>Faculdade de Medicina</t>
+    <t>Ciências da Saúde e Biológicas, Biologia, Biotecnologia, Ciências ambientais e marinhas</t>
+  </si>
+  <si>
+    <t>UMa - FCV</t>
   </si>
   <si>
     <t>Investigação marinha, Gestão ambiental, Ecoturismo</t>
@@ -521,397 +647,271 @@
     <t>Trabalho de campo intensivo, Biologia laboratorial</t>
   </si>
   <si>
-    <t>Ciências da Saúde e Biológicas, Investigação médica, Clínico, Hospitais universitários, Ciências da vida</t>
+    <t>Ciências da Saúde e Biológicas, Enfermagem, Tecnologias de saúde, Prática clínica</t>
+  </si>
+  <si>
+    <t>UMa - ESS</t>
   </si>
   <si>
     <t>Contributo crucial para a sustentabilidade do planeta, trabalho no terreno e contacto direto com a natureza.</t>
   </si>
   <si>
-    <t>UC - FMUC</t>
+    <t>Universidade de Lisboa</t>
+  </si>
+  <si>
+    <t>Instituto Superior Técnico (IST)</t>
   </si>
   <si>
     <t>Vagas de investigação pública limitadas, dependência de financiamento para bolsas e projetos científicos.</t>
   </si>
   <si>
+    <t>Engenharia e Tecnologias, Ciências Exatas e Tecnologias, Engenharia Aeroespacial, Inovação, R&amp;D</t>
+  </si>
+  <si>
+    <t>ULisboa - IST</t>
+  </si>
+  <si>
     <t>O trabalho é maioritariamente de laboratório/escritório ou existe forte componente prática no mar logo nos primeiros anos?</t>
   </si>
   <si>
+    <t>Ciências da Saúde e Biológicas, Investigação médica, Clínico, Saúde humana, Laboratorial</t>
+  </si>
+  <si>
+    <t>ULisboa - FM</t>
+  </si>
+  <si>
     <t>Artes, Património e Agricultura</t>
   </si>
   <si>
-    <t>Gestão e Economia, Ciências Sociais e Comunicação, Sociologia, Relações internacionais, Finanças</t>
-  </si>
-  <si>
     <t>Preservação histórica, agronomia e tradição</t>
   </si>
   <si>
-    <t>UC - FEUC</t>
+    <t>Direito e Políticas Públicas, Ciências Empresariais e Direito, Justiça, Regulamentação, Advocacia</t>
   </si>
   <si>
     <t>Gestão de património, Técnicas agrícolas, História da arte</t>
   </si>
   <si>
+    <t>ULisboa - FD</t>
+  </si>
+  <si>
     <t>Gestão agrícola, Museus, Conservação e restauro</t>
   </si>
   <si>
-    <t>Faculdade de Psicologia e de Ciências da Educação</t>
+    <t>Humanidades e Letras, Línguas, Cultura, História, Pensamento crítico, Ensino, Tradução</t>
+  </si>
+  <si>
+    <t>ULisboa - FL</t>
   </si>
   <si>
     <t>Aprendizagem imersiva no terreno e em laboratórios de restauro</t>
   </si>
   <si>
+    <t>Faculdade de Arquitetura</t>
+  </si>
+  <si>
     <t>Valorização das tradições, do território e do património cultural/agrícola nacional.</t>
   </si>
   <si>
-    <t>Psicologia e Ciências da Educação, Comportamento humano, Diagnóstico comportamental, Pedagogia</t>
-  </si>
-  <si>
-    <t>UC - FPCEUC</t>
+    <t>Arquitetura e Urbanismo, Tecnologias e Design, Design de espaços, Modelação 3D, Planeamento urbano</t>
+  </si>
+  <si>
+    <t>ULisboa - FA</t>
   </si>
   <si>
     <t>Recursos financeiros limitados no setor público (museus, conservação) e forte sazonalidade agrícola.</t>
   </si>
   <si>
+    <t>ISEG - Economia e Gestão</t>
+  </si>
+  <si>
     <t>Quais são as saídas na área agrícola ligadas à inovação tecnológica (AgTech) e agricultura de precisão?</t>
   </si>
   <si>
-    <t>Faculdade de Farmácia</t>
+    <t>Gestão e Economia, Ciências Empresariais e Direito, Finanças, Mercados, Liderança corporativa</t>
+  </si>
+  <si>
+    <t>ULisboa - ISEG</t>
+  </si>
+  <si>
+    <t>ISCSP - Ciências Sociais e Políticas</t>
+  </si>
+  <si>
+    <t>Ciências Sociais e Comunicação, Políticas Públicas, Media, Estratégia social, Recursos Humanos</t>
+  </si>
+  <si>
+    <t>ULisboa - ISCSP</t>
   </si>
   <si>
     <t>Ciências Empresariais e Direito</t>
   </si>
   <si>
-    <t>Ciências da Saúde e Biológicas, Ciências Farmacêuticas, Investigação laboratorial, Medicamentos</t>
+    <t>Faculdade de Psicologia</t>
   </si>
   <si>
     <t>Liderança corporativa e ética nos negócios</t>
   </si>
   <si>
-    <t>UC - FFUC</t>
+    <t>Psicologia e Ciências da Educação, Comportamento humano, Diagnóstico comportamental, Empatia</t>
   </si>
   <si>
     <t>Governança, Gestão estratégica, Direito empresarial</t>
   </si>
   <si>
+    <t>ULisboa - FP</t>
+  </si>
+  <si>
     <t>Corporações multinacionais, Banca, Advocacia de negócios</t>
   </si>
   <si>
-    <t>Faculdade de Ciências do Desporto e Educação Física</t>
+    <t>Faculdade de Ciências</t>
   </si>
   <si>
     <t>Casos práticos reais, Foco em network e apresentações</t>
   </si>
   <si>
+    <t>Ciências Exatas e Tecnologias, Ciências do Mar e Ambiente, Biologia, Computação, Matemática</t>
+  </si>
+  <si>
+    <t>ULisboa - Ciências</t>
+  </si>
+  <si>
     <t>Visão transversal do funcionamento das empresas, excelentes oportunidades em multinacionais e banca.</t>
   </si>
   <si>
-    <t>Psicologia e Ciências da Educação, Desporto, Atividade física, Bem-estar, Motricidade</t>
-  </si>
-  <si>
-    <t>UC - FCDEF</t>
-  </si>
-  <si>
     <t>Ambiente altamente competitivo e corporativo, exigência de disponibilidade total.</t>
   </si>
   <si>
+    <t>Faculdade de Medicina Veterinária</t>
+  </si>
+  <si>
     <t>O curso cruza efetivamente as duas áreas (Gestão + Direito) ou foca-se essencialmente numa delas com cadeiras isoladas da outra?</t>
   </si>
   <si>
-    <t>Escola Superior de Enfermagem</t>
+    <t>Ciências da Saúde e Biológicas, Artes, Património e Agricultura, Veterinária, Zootecnia</t>
+  </si>
+  <si>
+    <t>ULisboa - FMV</t>
+  </si>
+  <si>
+    <t>Ciências da Saúde e Biológicas, Ciências Farmacêuticas, Investigação laboratorial, Química aplicada</t>
   </si>
   <si>
     <t>Artes Cinematográficas e Media Digitais</t>
   </si>
   <si>
+    <t>ULisboa - FF</t>
+  </si>
+  <si>
     <t>Produção audiovisual, cinema e novas plataformas</t>
   </si>
   <si>
-    <t>Ciências da Saúde e Biológicas, Enfermagem, Cuidados de saúde, Prática clínica</t>
+    <t>Faculdade de Belas-Artes</t>
   </si>
   <si>
     <t>Realização, Edição de vídeo, Guionismo, Produção</t>
   </si>
   <si>
-    <t>UC - ESEFDUC</t>
-  </si>
-  <si>
     <t>Indústria do cinema, Televisão, Agências de publicidade</t>
   </si>
   <si>
-    <t>Universidade de Évora</t>
+    <t>Artes, Património e Agricultura, Tecnologias e Design, Pintura, Escultura, Design de comunicação</t>
+  </si>
+  <si>
+    <t>ULisboa - FBAUL</t>
   </si>
   <si>
     <t>Prática direta com equipamentos profissionais, Rodagens</t>
   </si>
   <si>
-    <t>Escola de Ciências e Tecnologia</t>
+    <t>Faculdade de Motricidade Humana</t>
   </si>
   <si>
     <t>Liberdade criativa, trabalho em projetos dinâmicos e visibilidade cultural dos conteúdos criados.</t>
   </si>
   <si>
-    <t>Ciências Exatas e Tecnologias, Engenharia e Tecnologias, Ciências do Mar e Ambiente, Energias</t>
-  </si>
-  <si>
-    <t>Mercado altamente informal em Portugal, precariedade laboral inicial e necessidade de investimento em equipamento.</t>
-  </si>
-  <si>
-    <t>UEvora - ECT</t>
+    <t>Psicologia e Ciências da Educação, Desporto, Reabilitação, Ergonomia, Movimento humano</t>
+  </si>
+  <si>
+    <t>ULisboa - FMH</t>
+  </si>
+  <si>
+    <t>Mercado com forte componente informal em Portugal, precariedade laboral inicial e necessidade de investimento em equipamento.</t>
+  </si>
+  <si>
+    <t>Instituto Superior de Agronomia</t>
+  </si>
+  <si>
+    <t>Artes, Património e Agricultura, Ciências do Mar e Ambiente, Engenharia agronómica, Florestas</t>
   </si>
   <si>
     <t>As escolas fornecem acesso a câmaras, estúdios e ilhas de edição profissionais durante os projetos académicos?</t>
   </si>
   <si>
-    <t>Escola de Ciências Sociais</t>
+    <t>ULisboa - ISA</t>
+  </si>
+  <si>
+    <t>Universidade do Minho</t>
+  </si>
+  <si>
+    <t>Escola de Engenharia</t>
+  </si>
+  <si>
+    <t>Engenharia e Tecnologias, Tecnologias e Design, Sistemas, Automação, Desenvolvimento de produto</t>
+  </si>
+  <si>
+    <t>UMinho - EE</t>
   </si>
   <si>
     <t>Psicologia e Ciências da Educação</t>
   </si>
   <si>
-    <t>Ciências Sociais e Comunicação, Humanidades e Letras, Gestão e Economia, Sociologia, Educação</t>
-  </si>
-  <si>
-    <t>UEvora - ECS</t>
-  </si>
-  <si>
-    <t>Escola de Artes</t>
-  </si>
-  <si>
-    <t>Artes, Património e Agricultura, Arquitetura e Urbanismo, Conservação e restauro, Design, Belas-Artes</t>
-  </si>
-  <si>
-    <t>UEvora - EA</t>
-  </si>
-  <si>
-    <t>Escola de Saúde e Desenvolvimento Humano</t>
-  </si>
-  <si>
-    <t>Ciências da Saúde e Biológicas, Psicologia e Ciências da Educação, Enfermagem, Saúde, Bem-estar</t>
-  </si>
-  <si>
-    <t>UEvora - ESDH</t>
-  </si>
-  <si>
-    <t>Universidade da Madeira</t>
-  </si>
-  <si>
-    <t>Faculdade de Ciências Exatas e da Engenharia</t>
-  </si>
-  <si>
-    <t>Engenharia e Tecnologias, Ciências Exatas e Tecnologias, Matemática, Computação, Engenharia</t>
-  </si>
-  <si>
-    <t>UMa - FCEE</t>
-  </si>
-  <si>
-    <t>Faculdade de Artes e Humanidades</t>
-  </si>
-  <si>
-    <t>Humanidades e Letras, Artes, Património e Agricultura, Línguas, Cultura e turismo insular</t>
-  </si>
-  <si>
-    <t>UMa - FAH</t>
-  </si>
-  <si>
-    <t>Faculdade de Ciências Sociais</t>
-  </si>
-  <si>
-    <t>Ciências Sociais e Comunicação, Gestão e Economia, Psicologia e Ciências da Educação, Direito</t>
-  </si>
-  <si>
-    <t>UMa - FCS</t>
-  </si>
-  <si>
-    <t>Faculdade de Ciências da Vida</t>
+    <t>Escola de Psicologia</t>
   </si>
   <si>
     <t>Compreensão do comportamento humano e ensino</t>
   </si>
   <si>
-    <t>Ciências da Saúde e Biológicas, Biologia, Biotecnologia, Ciências ambientais e marinhas</t>
+    <t>Psicologia e Ciências da Educação, Comportamento, Neurociência, Intervenção psicológica</t>
+  </si>
+  <si>
+    <t>UMinho - EPsi</t>
   </si>
   <si>
     <t>Empatia, Escuta ativa, Diagnóstico comportamental, Pedagogia</t>
   </si>
   <si>
-    <t>UMa - FCV</t>
+    <t>Escola de Economia e Gestão</t>
   </si>
   <si>
     <t>Clínico, Escolas, Recursos Humanos, Psicopedagogia</t>
   </si>
   <si>
+    <t>Gestão e Economia, Ciências Empresariais e Direito, Finanças, Negócios internacionais</t>
+  </si>
+  <si>
     <t>Prática clínica simulada, Estágios curriculares precoces</t>
   </si>
   <si>
+    <t>UMinho - EEG</t>
+  </si>
+  <si>
     <t>Enorme gratificação pessoal ao ajudar o próximo, alta utilidade prática em qualquer contexto organizacional.</t>
   </si>
   <si>
+    <t>Instituto de Educação</t>
+  </si>
+  <si>
+    <t>Psicologia e Ciências da Educação, Ciências Sociais e Comunicação, Pedagogia, Ensino</t>
+  </si>
+  <si>
     <t>Processo longo até à autonomia clínica (necessidade de estágio e inscrição na Ordem), carga emocional pesada.</t>
   </si>
   <si>
-    <t>Ciências da Saúde e Biológicas, Enfermagem, Tecnologias de saúde, Prática clínica</t>
-  </si>
-  <si>
-    <t>UMa - ESS</t>
+    <t>UMinho - IE</t>
   </si>
   <si>
     <t>O curso foca-se mais na vertente clínica, educacional ou de recursos humanos nas empresas?</t>
-  </si>
-  <si>
-    <t>Universidade de Lisboa</t>
-  </si>
-  <si>
-    <t>Instituto Superior Técnico (IST)</t>
-  </si>
-  <si>
-    <t>Engenharia e Tecnologias, Ciências Exatas e Tecnologias, Engenharia Aeroespacial, Inovação, R&amp;D</t>
-  </si>
-  <si>
-    <t>ULisboa - IST</t>
-  </si>
-  <si>
-    <t>Ciências da Saúde e Biológicas, Investigação médica, Clínico, Saúde humana, Laboratorial</t>
-  </si>
-  <si>
-    <t>ULisboa - FM</t>
-  </si>
-  <si>
-    <t>Direito e Políticas Públicas, Ciências Empresariais e Direito, Justiça, Regulamentação, Advocacia</t>
-  </si>
-  <si>
-    <t>ULisboa - FD</t>
-  </si>
-  <si>
-    <t>Humanidades e Letras, Línguas, Cultura, História, Pensamento crítico, Ensino, Tradução</t>
-  </si>
-  <si>
-    <t>ULisboa - FL</t>
-  </si>
-  <si>
-    <t>Faculdade de Arquitetura</t>
-  </si>
-  <si>
-    <t>Arquitetura e Urbanismo, Tecnologias e Design, Design de espaços, Modelação 3D, Planeamento urbano</t>
-  </si>
-  <si>
-    <t>ULisboa - FA</t>
-  </si>
-  <si>
-    <t>ISEG - Economia e Gestão</t>
-  </si>
-  <si>
-    <t>Gestão e Economia, Ciências Empresariais e Direito, Finanças, Mercados, Liderança corporativa</t>
-  </si>
-  <si>
-    <t>ULisboa - ISEG</t>
-  </si>
-  <si>
-    <t>ISCSP - Ciências Sociais e Políticas</t>
-  </si>
-  <si>
-    <t>Ciências Sociais e Comunicação, Políticas Públicas, Media, Estratégia social, Recursos Humanos</t>
-  </si>
-  <si>
-    <t>ULisboa - ISCSP</t>
-  </si>
-  <si>
-    <t>Faculdade de Psicologia</t>
-  </si>
-  <si>
-    <t>Psicologia e Ciências da Educação, Comportamento humano, Diagnóstico comportamental, Empatia</t>
-  </si>
-  <si>
-    <t>ULisboa - FP</t>
-  </si>
-  <si>
-    <t>Faculdade de Ciências</t>
-  </si>
-  <si>
-    <t>Ciências Exatas e Tecnologias, Ciências do Mar e Ambiente, Biologia, Computação, Matemática</t>
-  </si>
-  <si>
-    <t>ULisboa - Ciências</t>
-  </si>
-  <si>
-    <t>Faculdade de Medicina Veterinária</t>
-  </si>
-  <si>
-    <t>Ciências da Saúde e Biológicas, Artes, Património e Agricultura, Veterinária, Zootecnia</t>
-  </si>
-  <si>
-    <t>ULisboa - FMV</t>
-  </si>
-  <si>
-    <t>Ciências da Saúde e Biológicas, Ciências Farmacêuticas, Investigação laboratorial, Química aplicada</t>
-  </si>
-  <si>
-    <t>ULisboa - FF</t>
-  </si>
-  <si>
-    <t>Faculdade de Belas-Artes</t>
-  </si>
-  <si>
-    <t>Artes, Património e Agricultura, Tecnologias e Design, Pintura, Escultura, Design de comunicação</t>
-  </si>
-  <si>
-    <t>ULisboa - FBAUL</t>
-  </si>
-  <si>
-    <t>Faculdade de Motricidade Humana</t>
-  </si>
-  <si>
-    <t>Psicologia e Ciências da Educação, Desporto, Reabilitação, Ergonomia, Movimento humano</t>
-  </si>
-  <si>
-    <t>ULisboa - FMH</t>
-  </si>
-  <si>
-    <t>Instituto Superior de Agronomia</t>
-  </si>
-  <si>
-    <t>Artes, Património e Agricultura, Ciências do Mar e Ambiente, Engenharia agronómica, Florestas</t>
-  </si>
-  <si>
-    <t>ULisboa - ISA</t>
-  </si>
-  <si>
-    <t>Universidade do Minho</t>
-  </si>
-  <si>
-    <t>Escola de Engenharia</t>
-  </si>
-  <si>
-    <t>Engenharia e Tecnologias, Tecnologias e Design, Sistemas, Automação, Desenvolvimento de produto</t>
-  </si>
-  <si>
-    <t>UMinho - EE</t>
-  </si>
-  <si>
-    <t>Escola de Psicologia</t>
-  </si>
-  <si>
-    <t>Psicologia e Ciências da Educação, Comportamento, Neurociência, Intervenção psicológica</t>
-  </si>
-  <si>
-    <t>UMinho - EPsi</t>
-  </si>
-  <si>
-    <t>Escola de Economia e Gestão</t>
-  </si>
-  <si>
-    <t>Gestão e Economia, Ciências Empresariais e Direito, Finanças, Negócios internacionais</t>
-  </si>
-  <si>
-    <t>UMinho - EEG</t>
-  </si>
-  <si>
-    <t>Instituto de Educação</t>
-  </si>
-  <si>
-    <t>Psicologia e Ciências da Educação, Ciências Sociais e Comunicação, Pedagogia, Ensino</t>
-  </si>
-  <si>
-    <t>UMinho - IE</t>
   </si>
   <si>
     <t>Escola de Ciências</t>
@@ -1318,7 +1318,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1328,8 +1328,12 @@
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1568,415 +1572,432 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="E1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>21</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+      <c r="P1" s="3"/>
+      <c r="Q1" s="3"/>
+      <c r="R1" s="3"/>
+      <c r="S1" s="3"/>
+      <c r="T1" s="3"/>
+      <c r="U1" s="3"/>
+      <c r="V1" s="3"/>
+      <c r="W1" s="3"/>
+      <c r="X1" s="3"/>
+      <c r="Y1" s="3"/>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="3" t="s">
+      <c r="A2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="G2" s="1" t="s">
+      <c r="C2" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>39</v>
+      <c r="E2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F3" s="1" t="s">
+      <c r="A3" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>52</v>
+      <c r="B3" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="F4" s="1" t="s">
+      <c r="A4" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>65</v>
+      <c r="B4" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="D5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F5" s="1" t="s">
+      <c r="B5" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="C5" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="H5" s="1" t="s">
-        <v>78</v>
+      <c r="D5" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="B6" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="H6" s="1" t="s">
+      <c r="C6" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>91</v>
       </c>
+      <c r="E6" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="H7" s="1" t="s">
+      <c r="A7" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>105</v>
       </c>
+      <c r="D7" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>118</v>
+      <c r="A8" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>133</v>
+      <c r="A9" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>149</v>
+      <c r="A10" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>160</v>
+      <c r="A11" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>173</v>
+      <c r="A12" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>186</v>
+      <c r="A13" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>200</v>
+      <c r="A14" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>215</v>
+      <c r="A15" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>243</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>247</v>
+      <c r="A16" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="17">
@@ -6934,52 +6955,52 @@
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>22</v>
@@ -6990,880 +7011,880 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>138</v>
+        <v>120</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>140</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>147</v>
+        <v>127</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>151</v>
+        <v>131</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>154</v>
+        <v>133</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>156</v>
+        <v>134</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>161</v>
+        <v>137</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>163</v>
+        <v>138</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>142</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>175</v>
+        <v>145</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>177</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>180</v>
+        <v>148</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>183</v>
+        <v>150</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>184</v>
+        <v>151</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>187</v>
+        <v>153</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>189</v>
+        <v>155</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>191</v>
+        <v>156</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>194</v>
+        <v>158</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>197</v>
+        <v>160</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>198</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>201</v>
+        <v>164</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>204</v>
+        <v>165</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>206</v>
+        <v>167</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="s">
-        <v>208</v>
+        <v>169</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>210</v>
+        <v>170</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>212</v>
+        <v>173</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>214</v>
+        <v>174</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="s">
-        <v>208</v>
+        <v>169</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>216</v>
+        <v>176</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>218</v>
+        <v>177</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>219</v>
+        <v>178</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="s">
-        <v>208</v>
+        <v>169</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>220</v>
+        <v>180</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>221</v>
+        <v>182</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>222</v>
+        <v>183</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="s">
-        <v>208</v>
+        <v>169</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>223</v>
+        <v>185</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>224</v>
+        <v>187</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>225</v>
+        <v>188</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="s">
-        <v>226</v>
+        <v>190</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>227</v>
+        <v>191</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>228</v>
+        <v>193</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="s">
-        <v>226</v>
+        <v>190</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>230</v>
+        <v>196</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>231</v>
+        <v>198</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>232</v>
+        <v>199</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="s">
-        <v>226</v>
+        <v>190</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>233</v>
+        <v>200</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>234</v>
+        <v>202</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>235</v>
+        <v>203</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="s">
-        <v>226</v>
+        <v>190</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>236</v>
+        <v>205</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>238</v>
+        <v>207</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>240</v>
+        <v>208</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="s">
-        <v>226</v>
+        <v>190</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>245</v>
+        <v>211</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>246</v>
+        <v>212</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="s">
-        <v>248</v>
+        <v>214</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>249</v>
+        <v>215</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>250</v>
+        <v>217</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>251</v>
+        <v>218</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="s">
-        <v>248</v>
+        <v>214</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>166</v>
+        <v>139</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>252</v>
+        <v>220</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>253</v>
+        <v>221</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="s">
-        <v>248</v>
+        <v>214</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>254</v>
+        <v>224</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>255</v>
+        <v>226</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="s">
-        <v>248</v>
+        <v>214</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>151</v>
+        <v>131</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>256</v>
+        <v>228</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>257</v>
+        <v>229</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="s">
-        <v>248</v>
+        <v>214</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>258</v>
+        <v>231</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>259</v>
+        <v>233</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>260</v>
+        <v>234</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="s">
-        <v>248</v>
+        <v>214</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>261</v>
+        <v>236</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>262</v>
+        <v>238</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>263</v>
+        <v>239</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="s">
-        <v>248</v>
+        <v>214</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>264</v>
+        <v>240</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>265</v>
+        <v>241</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>266</v>
+        <v>242</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="E45" s="1" t="s">
         <v>248</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="s">
-        <v>248</v>
+        <v>214</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>271</v>
+        <v>252</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>272</v>
+        <v>253</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="s">
-        <v>248</v>
+        <v>214</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>273</v>
+        <v>256</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>274</v>
+        <v>258</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>275</v>
+        <v>259</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="s">
-        <v>248</v>
+        <v>214</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>187</v>
+        <v>153</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>277</v>
+        <v>262</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="s">
-        <v>248</v>
+        <v>214</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>278</v>
+        <v>264</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="s">
-        <v>248</v>
+        <v>214</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="s">
-        <v>248</v>
+        <v>214</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>284</v>
+        <v>275</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="E53" s="1" t="s">
         <v>287</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>291</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D55" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="E55" s="1" t="s">
         <v>298</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>300</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D56" s="1" t="s">
         <v>301</v>
@@ -7880,7 +7901,7 @@
         <v>304</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D57" s="1" t="s">
         <v>305</v>
@@ -7894,10 +7915,10 @@
         <v>303</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D58" s="1" t="s">
         <v>307</v>
@@ -7911,10 +7932,10 @@
         <v>303</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D59" s="1" t="s">
         <v>309</v>
@@ -7928,10 +7949,10 @@
         <v>303</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D60" s="1" t="s">
         <v>311</v>
@@ -7948,7 +7969,7 @@
         <v>313</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="D61" s="1" t="s">
         <v>314</v>
@@ -7965,7 +7986,7 @@
         <v>316</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>317</v>
@@ -7982,7 +8003,7 @@
         <v>320</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D63" s="1" t="s">
         <v>321</v>
@@ -7996,10 +8017,10 @@
         <v>319</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>166</v>
+        <v>139</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="D64" s="1" t="s">
         <v>323</v>
@@ -8013,10 +8034,10 @@
         <v>319</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>258</v>
+        <v>231</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D65" s="1" t="s">
         <v>325</v>
@@ -8030,10 +8051,10 @@
         <v>319</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D66" s="1" t="s">
         <v>327</v>
@@ -8047,10 +8068,10 @@
         <v>319</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D67" s="1" t="s">
         <v>329</v>
@@ -8064,10 +8085,10 @@
         <v>319</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>180</v>
+        <v>148</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D68" s="1" t="s">
         <v>331</v>
@@ -8084,7 +8105,7 @@
         <v>333</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="D69" s="1" t="s">
         <v>334</v>
@@ -8101,7 +8122,7 @@
         <v>337</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="D70" s="1" t="s">
         <v>338</v>
@@ -8115,10 +8136,10 @@
         <v>336</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>210</v>
+        <v>170</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D71" s="1" t="s">
         <v>340</v>
@@ -8135,7 +8156,7 @@
         <v>342</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D72" s="1" t="s">
         <v>343</v>
@@ -8152,7 +8173,7 @@
         <v>346</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D73" s="1" t="s">
         <v>347</v>
@@ -8169,7 +8190,7 @@
         <v>350</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D74" s="1" t="s">
         <v>351</v>
@@ -8186,7 +8207,7 @@
         <v>353</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D75" s="1" t="s">
         <v>354</v>
@@ -8203,7 +8224,7 @@
         <v>357</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D76" s="1" t="s">
         <v>358</v>
@@ -8220,7 +8241,7 @@
         <v>360</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D77" s="1" t="s">
         <v>361</v>
@@ -8237,7 +8258,7 @@
         <v>364</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D78" s="1" t="s">
         <v>365</v>
@@ -8254,7 +8275,7 @@
         <v>368</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D79" s="1" t="s">
         <v>369</v>
@@ -8271,7 +8292,7 @@
         <v>371</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D80" s="1" t="s">
         <v>372</v>
@@ -8288,7 +8309,7 @@
         <v>375</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D81" s="1" t="s">
         <v>376</v>
@@ -8305,7 +8326,7 @@
         <v>379</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D82" s="1" t="s">
         <v>380</v>
@@ -8322,7 +8343,7 @@
         <v>383</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D83" s="1" t="s">
         <v>384</v>
@@ -8339,7 +8360,7 @@
         <v>383</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D84" s="1" t="s">
         <v>387</v>
@@ -8356,7 +8377,7 @@
         <v>390</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D85" s="1" t="s">
         <v>391</v>
@@ -8373,7 +8394,7 @@
         <v>394</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D86" s="1" t="s">
         <v>395</v>
@@ -8390,7 +8411,7 @@
         <v>398</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D87" s="1" t="s">
         <v>399</v>
@@ -8407,7 +8428,7 @@
         <v>402</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D88" s="1" t="s">
         <v>403</v>
@@ -8424,7 +8445,7 @@
         <v>406</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D89" s="1" t="s">
         <v>407</v>
@@ -8441,7 +8462,7 @@
         <v>410</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D90" s="1" t="s">
         <v>411</v>
@@ -8458,7 +8479,7 @@
         <v>414</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D91" s="1" t="s">
         <v>415</v>

</xml_diff>